<commit_message>
Add reinforced concrete footprint of the foundations
RC footprint = blinding area pulled back by the 10 cm blinding projection
measured on the plan. Shown in blue on the drawing and added to the table.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017e4N5joefabz8rqJc3HWS5
</commit_message>
<xml_diff>
--- a/blinding_area.xlsx
+++ b/blinding_area.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -472,13 +472,33 @@
         <v>203.65</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Reinforced concrete footprint (m²)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1901.05</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  = blinding area less its projection (m)</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>area enclosed by S-BLINDING LINE in the foundation plan (footings, ground beams, rafts)</t>
         </is>

</xml_diff>